<commit_message>
feat(buffett): filtre ETF a effet de levier + criteres de convergence DE
Exclut les ETF a effet de levier/inverse (volatility decay, non fiables en
backtest STARR) via leverage_filter.is_leveraged_product ; ajoute les
parametres de convergence du Differential Evolution (min/max generations,
tolerance, seeds, polish) dans config.py. Rafraichit le cache financials_by_company.
</commit_message>
<xml_diff>
--- a/backend/data/financials_by_company/000090.SZ.xlsx
+++ b/backend/data/financials_by_company/000090.SZ.xlsx
@@ -4092,187 +4092,187 @@
       </c>
       <c r="DG1" t="inlineStr">
         <is>
+          <t>corporateActions</t>
+        </is>
+      </c>
+      <c r="DH1" t="inlineStr">
+        <is>
+          <t>regularMarketTime</t>
+        </is>
+      </c>
+      <c r="DI1" t="inlineStr">
+        <is>
+          <t>epsTrailingTwelveMonths</t>
+        </is>
+      </c>
+      <c r="DJ1" t="inlineStr">
+        <is>
+          <t>epsForward</t>
+        </is>
+      </c>
+      <c r="DK1" t="inlineStr">
+        <is>
+          <t>fiftyDayAverageChange</t>
+        </is>
+      </c>
+      <c r="DL1" t="inlineStr">
+        <is>
+          <t>fiftyDayAverageChangePercent</t>
+        </is>
+      </c>
+      <c r="DM1" t="inlineStr">
+        <is>
+          <t>twoHundredDayAverageChange</t>
+        </is>
+      </c>
+      <c r="DN1" t="inlineStr">
+        <is>
+          <t>twoHundredDayAverageChangePercent</t>
+        </is>
+      </c>
+      <c r="DO1" t="inlineStr">
+        <is>
+          <t>sourceInterval</t>
+        </is>
+      </c>
+      <c r="DP1" t="inlineStr">
+        <is>
+          <t>exchangeDataDelayedBy</t>
+        </is>
+      </c>
+      <c r="DQ1" t="inlineStr">
+        <is>
+          <t>marketState</t>
+        </is>
+      </c>
+      <c r="DR1" t="inlineStr">
+        <is>
+          <t>cryptoTradeable</t>
+        </is>
+      </c>
+      <c r="DS1" t="inlineStr">
+        <is>
+          <t>shortName</t>
+        </is>
+      </c>
+      <c r="DT1" t="inlineStr">
+        <is>
+          <t>hasPrePostMarketData</t>
+        </is>
+      </c>
+      <c r="DU1" t="inlineStr">
+        <is>
+          <t>firstTradeDateMilliseconds</t>
+        </is>
+      </c>
+      <c r="DV1" t="inlineStr">
+        <is>
+          <t>regularMarketChange</t>
+        </is>
+      </c>
+      <c r="DW1" t="inlineStr">
+        <is>
+          <t>regularMarketDayRange</t>
+        </is>
+      </c>
+      <c r="DX1" t="inlineStr">
+        <is>
           <t>fullExchangeName</t>
         </is>
       </c>
-      <c r="DH1" t="inlineStr">
+      <c r="DY1" t="inlineStr">
         <is>
           <t>averageDailyVolume3Month</t>
         </is>
       </c>
-      <c r="DI1" t="inlineStr">
+      <c r="DZ1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekLowChange</t>
         </is>
       </c>
-      <c r="DJ1" t="inlineStr">
+      <c r="EA1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekLowChangePercent</t>
         </is>
       </c>
-      <c r="DK1" t="inlineStr">
+      <c r="EB1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekRange</t>
         </is>
       </c>
-      <c r="DL1" t="inlineStr">
+      <c r="EC1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekHighChange</t>
         </is>
       </c>
-      <c r="DM1" t="inlineStr">
+      <c r="ED1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekHighChangePercent</t>
         </is>
       </c>
-      <c r="DN1" t="inlineStr">
+      <c r="EE1" t="inlineStr">
         <is>
           <t>fiftyTwoWeekChangePercent</t>
         </is>
       </c>
-      <c r="DO1" t="inlineStr">
+      <c r="EF1" t="inlineStr">
         <is>
           <t>earningsTimestampStart</t>
         </is>
       </c>
-      <c r="DP1" t="inlineStr">
+      <c r="EG1" t="inlineStr">
         <is>
           <t>earningsTimestampEnd</t>
         </is>
       </c>
-      <c r="DQ1" t="inlineStr">
-        <is>
-          <t>epsTrailingTwelveMonths</t>
-        </is>
-      </c>
-      <c r="DR1" t="inlineStr">
-        <is>
-          <t>epsForward</t>
-        </is>
-      </c>
-      <c r="DS1" t="inlineStr">
-        <is>
-          <t>fiftyDayAverageChange</t>
-        </is>
-      </c>
-      <c r="DT1" t="inlineStr">
-        <is>
-          <t>fiftyDayAverageChangePercent</t>
-        </is>
-      </c>
-      <c r="DU1" t="inlineStr">
-        <is>
-          <t>twoHundredDayAverageChange</t>
-        </is>
-      </c>
-      <c r="DV1" t="inlineStr">
-        <is>
-          <t>twoHundredDayAverageChangePercent</t>
-        </is>
-      </c>
-      <c r="DW1" t="inlineStr">
-        <is>
-          <t>sourceInterval</t>
-        </is>
-      </c>
-      <c r="DX1" t="inlineStr">
-        <is>
-          <t>exchangeDataDelayedBy</t>
-        </is>
-      </c>
-      <c r="DY1" t="inlineStr">
-        <is>
-          <t>cryptoTradeable</t>
-        </is>
-      </c>
-      <c r="DZ1" t="inlineStr">
-        <is>
-          <t>shortName</t>
-        </is>
-      </c>
-      <c r="EA1" t="inlineStr">
+      <c r="EH1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="EI1" t="inlineStr">
+        <is>
+          <t>esgPopulated</t>
+        </is>
+      </c>
+      <c r="EJ1" t="inlineStr">
+        <is>
+          <t>regularMarketChangePercent</t>
+        </is>
+      </c>
+      <c r="EK1" t="inlineStr">
+        <is>
+          <t>regularMarketPrice</t>
+        </is>
+      </c>
+      <c r="EL1" t="inlineStr">
+        <is>
+          <t>exchange</t>
+        </is>
+      </c>
+      <c r="EM1" t="inlineStr">
+        <is>
+          <t>messageBoardId</t>
+        </is>
+      </c>
+      <c r="EN1" t="inlineStr">
+        <is>
+          <t>exchangeTimezoneName</t>
+        </is>
+      </c>
+      <c r="EO1" t="inlineStr">
+        <is>
+          <t>exchangeTimezoneShortName</t>
+        </is>
+      </c>
+      <c r="EP1" t="inlineStr">
+        <is>
+          <t>gmtOffSetMilliseconds</t>
+        </is>
+      </c>
+      <c r="EQ1" t="inlineStr">
         <is>
           <t>longName</t>
-        </is>
-      </c>
-      <c r="EB1" t="inlineStr">
-        <is>
-          <t>exchange</t>
-        </is>
-      </c>
-      <c r="EC1" t="inlineStr">
-        <is>
-          <t>messageBoardId</t>
-        </is>
-      </c>
-      <c r="ED1" t="inlineStr">
-        <is>
-          <t>exchangeTimezoneName</t>
-        </is>
-      </c>
-      <c r="EE1" t="inlineStr">
-        <is>
-          <t>exchangeTimezoneShortName</t>
-        </is>
-      </c>
-      <c r="EF1" t="inlineStr">
-        <is>
-          <t>gmtOffSetMilliseconds</t>
-        </is>
-      </c>
-      <c r="EG1" t="inlineStr">
-        <is>
-          <t>market</t>
-        </is>
-      </c>
-      <c r="EH1" t="inlineStr">
-        <is>
-          <t>esgPopulated</t>
-        </is>
-      </c>
-      <c r="EI1" t="inlineStr">
-        <is>
-          <t>marketState</t>
-        </is>
-      </c>
-      <c r="EJ1" t="inlineStr">
-        <is>
-          <t>regularMarketChangePercent</t>
-        </is>
-      </c>
-      <c r="EK1" t="inlineStr">
-        <is>
-          <t>regularMarketPrice</t>
-        </is>
-      </c>
-      <c r="EL1" t="inlineStr">
-        <is>
-          <t>corporateActions</t>
-        </is>
-      </c>
-      <c r="EM1" t="inlineStr">
-        <is>
-          <t>regularMarketTime</t>
-        </is>
-      </c>
-      <c r="EN1" t="inlineStr">
-        <is>
-          <t>hasPrePostMarketData</t>
-        </is>
-      </c>
-      <c r="EO1" t="inlineStr">
-        <is>
-          <t>firstTradeDateMilliseconds</t>
-        </is>
-      </c>
-      <c r="EP1" t="inlineStr">
-        <is>
-          <t>regularMarketChange</t>
-        </is>
-      </c>
-      <c r="EQ1" t="inlineStr">
-        <is>
-          <t>regularMarketDayRange</t>
         </is>
       </c>
       <c r="ER1" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Shenzhen Tagen Group Co., Ltd. primarily engages in the urban construction, comprehensive development, and urban service businesses in China. The company's urban construction business includes municipal roads, municipal pipe networks, bridges and tunnels, and other urban infrastructure; water environment, landscaping, street lights, highways, and other projects; industrial and civil construction projects, earthwork, foundation and foundation engineering, and other construction projects; and rail transit projects and other fields. It also develops real estate projects, including mid-to-high-end residences, affordable housing, office buildings, hotels, urban complexes, industrial parks, etc. In addition, the company provides engineering construction, property management and leasing, and commercial operations and services; and urban infrastructure management and maintenance services, first-level land preparation services, commercial operation services, property services, etc. Further, it is involved in the engineering general contracting (EPC), construction general contracting, and other models; project management services, cultural venues management services, etc.; and civil engineering construction. The company was formerly known as Shenzhen Tonge (Group) Co., Ltd. Shenzhen Tagen Group Co., Ltd. was founded in 1988 and is headquartered in Shenzhen, China.</t>
+          <t>Shenzhen Tagen Group Co., Ltd. primarily engages in the urban construction, comprehensive development, and urban service businesses in China. The company engages in highway construction, industrial and civil building construction, earthwork, foundation engineering, and rail transit engineering; municipal public works construction, including municipal engineering, highways, bridges, building construction, electromechanical installation, water conservancy and hydropower. It also develops real estate projects, including mid-to-high-end residences, affordable housing, office buildings, hotels, urban complexes, industrial parks, etc. Further, it is involved in the engineering general contracting (EPC), construction general contracting, and other models; project management services, and civil engineering construction. The company was formerly known as Shenzhen Tonge (Group) Co., Ltd. Shenzhen Tagen Group Co., Ltd. was founded in 1983 and is headquartered in Shenzhen, China.</t>
         </is>
       </c>
       <c r="P2" t="n">
@@ -4377,34 +4377,34 @@
         <v>4</v>
       </c>
       <c r="U2" t="n">
-        <v>3.39</v>
+        <v>3.05</v>
       </c>
       <c r="V2" t="n">
-        <v>3.44</v>
+        <v>3.21</v>
       </c>
       <c r="W2" t="n">
-        <v>3.2</v>
+        <v>3.05</v>
       </c>
       <c r="X2" t="n">
-        <v>3.4</v>
+        <v>3.11</v>
       </c>
       <c r="Y2" t="n">
-        <v>3.39</v>
+        <v>3.05</v>
       </c>
       <c r="Z2" t="n">
-        <v>3.44</v>
+        <v>3.21</v>
       </c>
       <c r="AA2" t="n">
-        <v>3.2</v>
+        <v>3.05</v>
       </c>
       <c r="AB2" t="n">
-        <v>3.4</v>
+        <v>3.11</v>
       </c>
       <c r="AC2" t="n">
         <v>0.1</v>
       </c>
       <c r="AD2" t="n">
-        <v>3</v>
+        <v>3.28</v>
       </c>
       <c r="AE2" t="n">
         <v>1752192000</v>
@@ -4413,37 +4413,37 @@
         <v>2.8249</v>
       </c>
       <c r="AG2" t="n">
-        <v>5.69</v>
+        <v>5.64</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.591</v>
+        <v>0.613</v>
       </c>
       <c r="AI2" t="n">
-        <v>83.25</v>
+        <v>77.25</v>
       </c>
       <c r="AJ2" t="n">
-        <v>6.1666665</v>
+        <v>5.722222</v>
       </c>
       <c r="AK2" t="n">
-        <v>30587731</v>
+        <v>16388360</v>
       </c>
       <c r="AL2" t="n">
-        <v>30587731</v>
+        <v>16388360</v>
       </c>
       <c r="AM2" t="n">
-        <v>29719475</v>
+        <v>29182936</v>
       </c>
       <c r="AN2" t="n">
-        <v>40812729</v>
+        <v>20857765</v>
       </c>
       <c r="AO2" t="n">
-        <v>40812729</v>
+        <v>20857765</v>
       </c>
       <c r="AP2" t="n">
-        <v>3.32</v>
+        <v>3.08</v>
       </c>
       <c r="AQ2" t="n">
-        <v>3.33</v>
+        <v>3.09</v>
       </c>
       <c r="AR2" t="n">
         <v>0</v>
@@ -4452,13 +4452,13 @@
         <v>0</v>
       </c>
       <c r="AT2" t="n">
-        <v>6222256128</v>
+        <v>5773805056</v>
       </c>
       <c r="AU2" t="n">
-        <v>6334369021</v>
+        <v>5773805391</v>
       </c>
       <c r="AV2" t="n">
-        <v>3.18</v>
+        <v>2.98</v>
       </c>
       <c r="AW2" t="n">
         <v>4.88</v>
@@ -4470,19 +4470,19 @@
         <v>0.86025</v>
       </c>
       <c r="AZ2" t="n">
-        <v>0.26698336</v>
+        <v>0.24774133</v>
       </c>
       <c r="BA2" t="n">
-        <v>3.5282</v>
+        <v>3.4424</v>
       </c>
       <c r="BB2" t="n">
-        <v>3.75805</v>
+        <v>3.73285</v>
       </c>
       <c r="BC2" t="n">
         <v>0.036</v>
       </c>
       <c r="BD2" t="n">
-        <v>0.010619468</v>
+        <v>0.011803279</v>
       </c>
       <c r="BE2" t="inlineStr">
         <is>
@@ -4493,13 +4493,13 @@
         <v>0</v>
       </c>
       <c r="BG2" t="n">
-        <v>14041564160</v>
+        <v>13593112576</v>
       </c>
       <c r="BH2" t="n">
         <v>0.00686</v>
       </c>
       <c r="BI2" t="n">
-        <v>1113279370</v>
+        <v>1106384437</v>
       </c>
       <c r="BJ2" t="n">
         <v>1868545434</v>
@@ -4508,7 +4508,7 @@
         <v>0.41724998</v>
       </c>
       <c r="BL2" t="n">
-        <v>0.03694</v>
+        <v>0.03692</v>
       </c>
       <c r="BM2" t="n">
         <v>1868545434</v>
@@ -4517,7 +4517,7 @@
         <v>6.018</v>
       </c>
       <c r="BO2" t="n">
-        <v>0.55333996</v>
+        <v>0.5134596</v>
       </c>
       <c r="BP2" t="n">
         <v>1767139200</v>
@@ -4546,16 +4546,16 @@
         <v>1560988800</v>
       </c>
       <c r="BX2" t="n">
-        <v>0.602</v>
+        <v>0.583</v>
       </c>
       <c r="BY2" t="n">
-        <v>15.689</v>
+        <v>15.188</v>
       </c>
       <c r="BZ2" t="n">
-        <v>-0.023054779</v>
+        <v>-0.1480447</v>
       </c>
       <c r="CA2" t="n">
-        <v>0.24487448</v>
+        <v>0.20116603</v>
       </c>
       <c r="CB2" t="n">
         <v>0.1</v>
@@ -4569,7 +4569,7 @@
         </is>
       </c>
       <c r="CE2" t="n">
-        <v>3.33</v>
+        <v>3.09</v>
       </c>
       <c r="CF2" t="inlineStr">
         <is>
@@ -4670,137 +4670,137 @@
       </c>
       <c r="DG2" t="inlineStr">
         <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="DH2" t="n">
+        <v>1783062249</v>
+      </c>
+      <c r="DI2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="DJ2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="DK2" t="n">
+        <v>-0.35240006</v>
+      </c>
+      <c r="DL2" t="n">
+        <v>-0.102370456</v>
+      </c>
+      <c r="DM2" t="n">
+        <v>-0.6428501599999999</v>
+      </c>
+      <c r="DN2" t="n">
+        <v>-0.1722143</v>
+      </c>
+      <c r="DO2" t="n">
+        <v>15</v>
+      </c>
+      <c r="DP2" t="n">
+        <v>15</v>
+      </c>
+      <c r="DQ2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="DR2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DS2" t="inlineStr">
+        <is>
+          <t>SHENZHEN TAGEN GROUP CO LTD</t>
+        </is>
+      </c>
+      <c r="DT2" t="b">
+        <v>0</v>
+      </c>
+      <c r="DU2" t="n">
+        <v>932520600000</v>
+      </c>
+      <c r="DV2" t="n">
+        <v>0.03999996</v>
+      </c>
+      <c r="DW2" t="inlineStr">
+        <is>
+          <t>3.05 - 3.11</t>
+        </is>
+      </c>
+      <c r="DX2" t="inlineStr">
+        <is>
           <t>Shenzhen</t>
         </is>
       </c>
-      <c r="DH2" t="n">
-        <v>29719475</v>
-      </c>
-      <c r="DI2" t="n">
-        <v>0.14999986</v>
-      </c>
-      <c r="DJ2" t="n">
-        <v>0.047169764</v>
-      </c>
-      <c r="DK2" t="inlineStr">
-        <is>
-          <t>3.18 - 4.88</t>
-        </is>
-      </c>
-      <c r="DL2" t="n">
-        <v>-1.5500002</v>
-      </c>
-      <c r="DM2" t="n">
-        <v>-0.317623</v>
-      </c>
-      <c r="DN2" t="n">
-        <v>-2.3054779</v>
-      </c>
-      <c r="DO2" t="n">
+      <c r="DY2" t="n">
+        <v>29182936</v>
+      </c>
+      <c r="DZ2" t="n">
+        <v>0.109999895</v>
+      </c>
+      <c r="EA2" t="n">
+        <v>0.036912717</v>
+      </c>
+      <c r="EB2" t="inlineStr">
+        <is>
+          <t>2.98 - 4.88</t>
+        </is>
+      </c>
+      <c r="EC2" t="n">
+        <v>-1.7900002</v>
+      </c>
+      <c r="ED2" t="n">
+        <v>-0.36680332</v>
+      </c>
+      <c r="EE2" t="n">
+        <v>-14.80447</v>
+      </c>
+      <c r="EF2" t="n">
         <v>1651229940</v>
       </c>
-      <c r="DP2" t="n">
+      <c r="EG2" t="n">
         <v>1651492800</v>
       </c>
-      <c r="DQ2" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="DR2" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="DS2" t="n">
-        <v>-0.19819999</v>
-      </c>
-      <c r="DT2" t="n">
-        <v>-0.05617595</v>
-      </c>
-      <c r="DU2" t="n">
-        <v>-0.42805004</v>
-      </c>
-      <c r="DV2" t="n">
-        <v>-0.11390217</v>
-      </c>
-      <c r="DW2" t="n">
-        <v>15</v>
-      </c>
-      <c r="DX2" t="n">
-        <v>15</v>
-      </c>
-      <c r="DY2" t="b">
+      <c r="EH2" t="inlineStr">
+        <is>
+          <t>cn_market</t>
+        </is>
+      </c>
+      <c r="EI2" t="b">
         <v>0</v>
       </c>
-      <c r="DZ2" t="inlineStr">
-        <is>
-          <t>SHENZHEN TAGEN GROUP CO LTD</t>
-        </is>
-      </c>
-      <c r="EA2" t="inlineStr">
+      <c r="EJ2" t="n">
+        <v>1.3114742</v>
+      </c>
+      <c r="EK2" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="EL2" t="inlineStr">
+        <is>
+          <t>SHZ</t>
+        </is>
+      </c>
+      <c r="EM2" t="inlineStr">
+        <is>
+          <t>finmb_6465470</t>
+        </is>
+      </c>
+      <c r="EN2" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
+        </is>
+      </c>
+      <c r="EO2" t="inlineStr">
+        <is>
+          <t>CST</t>
+        </is>
+      </c>
+      <c r="EP2" t="n">
+        <v>28800000</v>
+      </c>
+      <c r="EQ2" t="inlineStr">
         <is>
           <t>Shenzhen Tagen Group Co., Ltd.</t>
-        </is>
-      </c>
-      <c r="EB2" t="inlineStr">
-        <is>
-          <t>SHZ</t>
-        </is>
-      </c>
-      <c r="EC2" t="inlineStr">
-        <is>
-          <t>finmb_6465470</t>
-        </is>
-      </c>
-      <c r="ED2" t="inlineStr">
-        <is>
-          <t>Asia/Shanghai</t>
-        </is>
-      </c>
-      <c r="EE2" t="inlineStr">
-        <is>
-          <t>CST</t>
-        </is>
-      </c>
-      <c r="EF2" t="n">
-        <v>28800000</v>
-      </c>
-      <c r="EG2" t="inlineStr">
-        <is>
-          <t>cn_market</t>
-        </is>
-      </c>
-      <c r="EH2" t="b">
-        <v>0</v>
-      </c>
-      <c r="EI2" t="inlineStr">
-        <is>
-          <t>PREPRE</t>
-        </is>
-      </c>
-      <c r="EJ2" t="n">
-        <v>-1.7699168</v>
-      </c>
-      <c r="EK2" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="EL2" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="EM2" t="n">
-        <v>1782111885</v>
-      </c>
-      <c r="EN2" t="b">
-        <v>0</v>
-      </c>
-      <c r="EO2" t="n">
-        <v>932520600000</v>
-      </c>
-      <c r="EP2" t="n">
-        <v>-0.06000018</v>
-      </c>
-      <c r="EQ2" t="inlineStr">
-        <is>
-          <t>3.2 - 3.4</t>
         </is>
       </c>
       <c r="ER2" t="inlineStr"/>

</xml_diff>